<commit_message>
updates to message output variables and validation sheet to align with CORE-000029
</commit_message>
<xml_diff>
--- a/rules/CORE-000026/negative/01/data/unit-test-coreid-CG0468-negative.xlsx
+++ b/rules/CORE-000026/negative/01/data/unit-test-coreid-CG0468-negative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000026\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1268C477-755A-492B-A2D1-87818D21E34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3117144-E0DE-4FBF-B48A-85E24AE8E0C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="107">
   <si>
     <t>Product</t>
   </si>
@@ -336,6 +336,15 @@
   </si>
   <si>
     <t>Functional Tests</t>
+  </si>
+  <si>
+    <t>LBTPTNUM</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
+  </si>
+  <si>
+    <t>FTTPTNUM</t>
   </si>
 </sst>
 </file>
@@ -451,7 +460,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -472,7 +481,6 @@
     <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -487,6 +495,363 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="21">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -517,363 +882,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -888,27 +896,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7A374A5A-962A-44F7-9BBB-17BB7E5DB6DD}" name="Table1" displayName="Table1" ref="A1:S7" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="19" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7A374A5A-962A-44F7-9BBB-17BB7E5DB6DD}" name="Table1" displayName="Table1" ref="A1:S7" totalsRowShown="0" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="17">
   <autoFilter ref="A1:S7" xr:uid="{7A374A5A-962A-44F7-9BBB-17BB7E5DB6DD}"/>
   <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{90521441-BDCF-490B-94BE-9C373402EC6B}" name="STUDYID" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{9A9C517F-5212-404D-9045-5E2ADAF65497}" name="DOMAIN" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{B6962D9A-6030-446C-A5C8-96771D18EB0F}" name="USUBJID" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{DFA0638B-44BD-47AC-8D88-702BF038F0B6}" name="FTSEQ" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{32D18473-4056-473C-A7C3-A32475228286}" name="FTTESTCD" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{86842DE3-181F-4063-9D49-68F25A1930CB}" name="FTTEST" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{4F06D386-C603-4CBC-AED6-562063251C87}" name="FTCAT" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{98A15F80-9812-4C0E-B06B-757CECDE02B1}" name="FTSCAT" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{DCCF7160-0793-4769-9CE8-060A2BC8C650}" name="FTORRES" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{1E8659C9-3A1B-417F-B232-7D054E30FD1C}" name="FTSTRESC" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{90521441-BDCF-490B-94BE-9C373402EC6B}" name="STUDYID" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{9A9C517F-5212-404D-9045-5E2ADAF65497}" name="DOMAIN" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{B6962D9A-6030-446C-A5C8-96771D18EB0F}" name="USUBJID" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{DFA0638B-44BD-47AC-8D88-702BF038F0B6}" name="FTSEQ" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{32D18473-4056-473C-A7C3-A32475228286}" name="FTTESTCD" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{86842DE3-181F-4063-9D49-68F25A1930CB}" name="FTTEST" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{4F06D386-C603-4CBC-AED6-562063251C87}" name="FTCAT" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{98A15F80-9812-4C0E-B06B-757CECDE02B1}" name="FTSCAT" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{DCCF7160-0793-4769-9CE8-060A2BC8C650}" name="FTORRES" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{1E8659C9-3A1B-417F-B232-7D054E30FD1C}" name="FTSTRESC" dataDxfId="7"/>
     <tableColumn id="11" xr3:uid="{1035E300-BAEE-4B01-BC39-FBAC8135AE46}" name="FTSTRESN"/>
-    <tableColumn id="12" xr3:uid="{4A3DB5AF-AC3F-4810-9BD3-2AB5C1CB355A}" name="FTLOBXFL" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{EDCB795B-6074-4DCB-9D41-F47BFD3B380F}" name="FTREPNUM" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{AC19C88A-EF33-4B7F-9247-59BBF023E8A4}" name="VISITNUM" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{3462194F-FBA6-4DB3-9AB3-41DC0B209D45}" name="VISIT" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{E3BA55F8-06E5-44D7-9E30-91F70E338B46}" name="EPOCH" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{653B6DF3-002C-43B7-9332-1E0C034BFC81}" name="FTDTC" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{CCCBA374-A302-46BD-AF32-767C279CF3E8}" name="FTDY" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{4A3DB5AF-AC3F-4810-9BD3-2AB5C1CB355A}" name="FTLOBXFL" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{EDCB795B-6074-4DCB-9D41-F47BFD3B380F}" name="FTREPNUM" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{AC19C88A-EF33-4B7F-9247-59BBF023E8A4}" name="VISITNUM" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{3462194F-FBA6-4DB3-9AB3-41DC0B209D45}" name="VISIT" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{E3BA55F8-06E5-44D7-9E30-91F70E338B46}" name="EPOCH" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{653B6DF3-002C-43B7-9332-1E0C034BFC81}" name="FTDTC" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{CCCBA374-A302-46BD-AF32-767C279CF3E8}" name="FTDY" dataDxfId="0"/>
     <tableColumn id="19" xr3:uid="{A2A67044-EB0E-4146-B2CA-8C51D3777063}" name="FTTPT"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1263,7 +1271,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -1309,24 +1317,64 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="10">
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B4" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F4" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1727,61 +1775,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="M1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="P1" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="Q1" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="R1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="12" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1963,169 +2011,163 @@
       </c>
     </row>
     <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="10">
         <v>1</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="K5" s="10"/>
-      <c r="L5" s="11" t="s">
+      <c r="L5" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="M5" s="11">
+      <c r="M5" s="10">
         <v>1</v>
       </c>
-      <c r="N5" s="11">
+      <c r="N5" s="10">
         <v>2</v>
       </c>
-      <c r="O5" s="11" t="s">
+      <c r="O5" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="P5" s="11" t="s">
+      <c r="P5" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q5" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="R5" s="11">
+      <c r="R5" s="10">
         <v>-2</v>
       </c>
-      <c r="S5" s="10"/>
     </row>
     <row r="6" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="10">
         <v>2</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="K6" s="10"/>
-      <c r="L6" s="11" t="s">
+      <c r="L6" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="M6" s="11">
+      <c r="M6" s="10">
         <v>1</v>
       </c>
-      <c r="N6" s="11">
+      <c r="N6" s="10">
         <v>2</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="P6" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="Q6" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="R6" s="11">
+      <c r="R6" s="10">
         <v>-2</v>
       </c>
-      <c r="S6" s="10"/>
     </row>
     <row r="7" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="10">
         <v>3</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="K7" s="10"/>
-      <c r="L7" s="11" t="s">
+      <c r="L7" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="M7" s="11">
+      <c r="M7" s="10">
         <v>1</v>
       </c>
-      <c r="N7" s="11">
+      <c r="N7" s="10">
         <v>2</v>
       </c>
-      <c r="O7" s="11" t="s">
+      <c r="O7" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="P7" s="11" t="s">
+      <c r="P7" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="Q7" s="11" t="s">
+      <c r="Q7" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="R7" s="11">
+      <c r="R7" s="10">
         <v>-2</v>
       </c>
-      <c r="S7" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>